<commit_message>
🤖 Zapis ocen z www do Piwa.xlsx
</commit_message>
<xml_diff>
--- a/Piwa.xlsx
+++ b/Piwa.xlsx
@@ -589,6 +589,11 @@
           <t>https://ocen-piwo.pl/maryensztadt-summertime-papaja-mango-brzoskwinia-s1-n36566</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Dawid: 1</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="54.75" customHeight="1">
       <c r="A3" s="1" t="n">
@@ -625,6 +630,11 @@
           <t>.</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Dawid: 3</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="1" t="n">
@@ -661,6 +671,11 @@
           <t>https://ocen-piwo.pl/trzech-kumpli-lager-wiedenski-s1-n25855</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Dawid: 2</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="75" customHeight="1">
       <c r="A5" s="1">
@@ -698,6 +713,11 @@
           <t>https://ocen-piwo.pl/magic-road-mochi-green-s1-n33867</t>
         </is>
       </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Dawid: 3,5</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="1">
@@ -735,6 +755,11 @@
           <t>https://ocen-piwo.pl/gosciszewo-ogrod-mistrza-witbier-z-tymiankiem-cytrynowym-s1-n8343</t>
         </is>
       </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Dawid: 1,25</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="60" customHeight="1">
       <c r="A7" s="1">
@@ -772,6 +797,11 @@
           <t>https://ocen-piwo.pl/stu-mostow-berry-up-s1-n36564</t>
         </is>
       </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Dawid: 4,5</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="1">
@@ -809,6 +839,11 @@
           <t>https://browarpinta.pl/produkt/pinta-classics-mild/</t>
         </is>
       </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Dawid: 2</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="1">
@@ -846,6 +881,11 @@
           <t>https://ocen-piwo.pl/funky-fluid-gelato-purple-fluff-s1-n26711</t>
         </is>
       </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Dawid: 4</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="60" customHeight="1">
       <c r="A10" s="1">
@@ -883,6 +923,11 @@
           <t>https://browarpinta.pl/produkt/pinta-summer-beer-supply-polish-cold-ipa/</t>
         </is>
       </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Dawid: 1,25</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="60" customHeight="1">
       <c r="A11" s="1">
@@ -920,6 +965,11 @@
           <t>https://ocen-piwo.pl/nepomucen-smoothie-bowl-sweet-morning-s1-n33621</t>
         </is>
       </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Dawid: 2,5</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="75" customHeight="1">
       <c r="A12" s="1">
@@ -957,6 +1007,11 @@
           <t>https://ocen-piwo.pl/amber-po-godzinach-graff-apple-wheat-s1-n5590</t>
         </is>
       </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Dawid: 3</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="1">
@@ -994,6 +1049,11 @@
           <t>https://www.lidl.pl/p/za-miastem-wolny-wieczor/p10035546</t>
         </is>
       </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Dawid: 2</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="75" customHeight="1">
       <c r="A14" s="1">
@@ -1031,6 +1091,11 @@
           <t>https://ocen-piwo.pl/bojan-bananowe-s1-n29230</t>
         </is>
       </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Dawid: 2</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="60" customHeight="1">
       <c r="A15" s="1">
@@ -1068,6 +1133,11 @@
           <t>https://browarzakladowy.pl/sokowirowka-kwasne-ale-z-malinami-i-jagodami/</t>
         </is>
       </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Dawid: 1,5</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="1">
@@ -1105,6 +1175,11 @@
           <t>https://ocen-piwo.pl/funky-fluid-farm-to-glass-26-citra-s1-n36167</t>
         </is>
       </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Dawid: 2,5</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="1">
@@ -1142,6 +1217,11 @@
           <t>https://ocen-piwo.pl/zakladowy-hiszpanskie-wakacje-s1-n34316</t>
         </is>
       </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Dawid: 2,5</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="45" customHeight="1">
       <c r="A18" s="1">
@@ -1179,6 +1259,11 @@
           <t>https://browarzakladowy.pl/wyjac-grilla-to-jest-chwila-new-zealand-west-coast-ipa/</t>
         </is>
       </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Dawid: 2</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="1" t="n">
@@ -1213,6 +1298,11 @@
       <c r="H19" s="1" t="inlineStr">
         <is>
           <t>https://ocen-piwo.pl/litovel-cerny-citron-s1-n3209</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Dawid: 4</t>
         </is>
       </c>
     </row>

</xml_diff>